<commit_message>
feat: aggiungi Manuel Locatelli (Juventus, n.5) + foto SortItOutSi
</commit_message>
<xml_diff>
--- a/data/sots_overrides.xlsx
+++ b/data/sots_overrides.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -624,6 +624,18 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Manuel Locatelli</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/43167354/manuel-locatelli</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: 16 nuovi override SOTS (foto FM26) per giocatori esteri
Aggiunti override manuali in data/sots_overrides.xlsx per 16 giocatori che
find_more_sots_matches non riusciva a matchare automaticamente (translitterazioni
o slug SOTS molto diversi dal nome TM/PID):

- Antoine Sekongo, Baptiste Mouazan, Emersonn, Emiliano Filippis,
  Ewen Jaouen, Gessime Yassine, Ibrahim El Kadiri, Jeremy Monga,
  Joseph Kalulu, Lucas Stassin, Martial Tia, Triston Rowe,
  Victor Munoz, Wisdom Amey, Yann Gboho, Yassine Benhattab

Workflow seguito (come da diario 6 mag):
1. Aggiunte 16 righe a data/sots_overrides.xlsx (totale 33 override storici)
2. python3 apply_sots_overrides.py: match per nome + download face + update JSON

Risultato:
- 16/16 foto SOTS scaricate in data/photos/players_sots_lookup/
- Campi sortitoutsi_person_id, sortitoutsi_face_url, sortitoutsi_profile_url,
  sortitoutsi_face_local_lookup popolati per tutti e 16
</commit_message>
<xml_diff>
--- a/data/sots_overrides.xlsx
+++ b/data/sots_overrides.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -636,6 +636,198 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Antoine Sekongo</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000279641/antoine-sekongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Baptiste Mouazan</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/49050068/baptiste-mouazan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Emersonn</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/19409149/emersonn</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Emiliano Filippis</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000047967/emiliano-filippis</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ewen Jaouen</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000183134/ewen-jaouen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Gessime Yassine</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000333625/gessime-yassine</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ibrahim El Kadiri</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/37075213/ibrahim-el-kadiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jeremy Monga</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000474101/jeremy-monga</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Joseph Kalulu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000402614/joseph-kalulu</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Lucas Stassin</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000022188/lucas-stassin</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Martial Tia</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/12095307/martial-tia</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Triston Rowe</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000283795/triston-rowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Víctor Muñoz</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000126470/victor-munoz</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wisdom Amey</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000097938/wisdom-amey</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Yann Gboho</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/49038961/yann-gboho</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Yassine Benhattab</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/49056530/yassine-benhattab</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>